<commit_message>
Regenerate all QA reports with Zout 5.9.1 WARN check and updated review system
All 16 reports rebuilt from source .ibs files using regen_all.py. New in this run:
- 5.9.1 Zout WARN entries now appear in the attention section with load-line plots
- Review keys use identity-only hashing (stable across tool updates)
- Fix proposal stubs present in HTML/JSON where applicable
- New iv_clamp_sweep_* SVG assets for Micron y32a, z41c, z41c_it
- k450_wlcsp/ report directory added (57 Zout WARNs, 2 fix proposals)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/ibis_files/hark_abi_gen3/hark_abi_gen3.xlsx
+++ b/reports/ibis_files/hark_abi_gen3/hark_abi_gen3.xlsx
@@ -116,7 +116,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-09T23:35:21-05:00</t>
+          <t>2026-06-12T22:46:15-05:00</t>
         </is>
       </c>
     </row>
@@ -256,7 +256,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7.2.1</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -266,8 +266,10 @@
           <t>Errors</t>
         </is>
       </c>
-      <c r="B16">
-        <v>0</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -276,8 +278,10 @@
           <t>Warnings</t>
         </is>
       </c>
-      <c r="B17">
-        <v>0</v>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -286,8 +290,10 @@
           <t>Cautions</t>
         </is>
       </c>
-      <c r="B18">
-        <v>0</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -298,7 +304,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>C:\Users\simom\Desktop\Projects\IBIS_QA\ibischk721_win_64\ibischk7_64.exe</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -349,7 +355,7 @@
         </is>
       </c>
       <c r="B25">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -359,7 +365,7 @@
         </is>
       </c>
       <c r="B26">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27">
@@ -423,14 +429,14 @@
           <t>IBIS file passes IBISCHK</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr" s="4">
-        <is>
-          <t>PASS</t>
+      <c r="D31" t="inlineStr" s="6">
+        <is>
+          <t>REVIEW</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>PASS=3. No existing '|IQ Score:' tag found inside the .ibs file. This is reported as a writeback note only; it does not fail the quality check because this tool is intended to help assign the score. | IBISCHK version not found documented inside the .ibs file. This is reported as a documentation note only; it does not block Level 1. | IBISCHK: 0 errors, 0 warning(s): IBISCHK path: C:\Users\simom\Desktop\Projects\IBIS_QA\ibischk721_win_64\ibischk7_64.exe</t>
+          <t>WARN=1, PASS=2. No existing '|IQ Score:' tag found inside the .ibs file. This is reported as a writeback note only; it does not fail the quality check because this tool is intended to help assign the score. | IBISCHK version not found documented inside the .ibs file. This is reported as a documentation note only; it does not block Level 1. | IBISCHK not found on PATH — skipping execution check. Install IBISCHK and ensure it is on PATH</t>
         </is>
       </c>
     </row>
@@ -8495,7 +8501,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2.1-file-abi_gen3.ibs-b71c7faa0d9f</t>
+          <t>2.1-file-abi_gen3.ibs-6399e563771f</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8562,7 +8568,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2.1-file-abi_gen3.ibs-359c853f7b08</t>
+          <t>2.1-file-abi_gen3.ibs-6399e563771f-2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8629,7 +8635,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2.1-file-abi_gen3.ibs-b418a8b55da6</t>
+          <t>2.1-file-abi_gen3.ibs-6399e563771f-3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8647,14 +8653,14 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr" s="4">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr" s="4">
-        <is>
-          <t>PASS</t>
+      <c r="E4" t="inlineStr" s="6">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="6">
+        <is>
+          <t>WARN</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -8684,19 +8690,19 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>IBISCHK: 0 errors, 0 warning(s)</t>
+          <t>IBISCHK not found on PATH — skipping execution check. Install IBISCHK and ensure it is on PATH.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>IBISCHK path: C:\Users\simom\Desktop\Projects\IBIS_QA\ibischk721_win_64\ibischk7_64.exe</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3.1.1-component-ABI_Serdes-7f344aca8484</t>
+          <t>3.1.1-component-ABI_Serdes-d86432829bb9</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8763,7 +8769,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3.1.2-component-ABI_Serdes-850f9687f203</t>
+          <t>3.1.2-component-ABI_Serdes-ec9208e585a7</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8830,7 +8836,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3.2.1-component-ABI_Serdes-f2a499e48d6e</t>
+          <t>3.2.1-component-ABI_Serdes-c385b7227034</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8897,7 +8903,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>4.1-file-abi_gen3.ibs-2d42db650860</t>
+          <t>4.1-file-abi_gen3.ibs-6a83d0d7fdae</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8964,7 +8970,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3.2.2-component-ABI_Serdes-d3e4fb5f987a</t>
+          <t>3.2.2-component-ABI_Serdes-12512cb97d3e</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9036,7 +9042,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3.3.1-component-ABI_Serdes-f7dc70ed79fd</t>
+          <t>3.3.1-component-ABI_Serdes-288a3bf98f97</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -9103,7 +9109,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3.3.2-component-ABI_Serdes-47223426b5c7</t>
+          <t>3.3.2-component-ABI_Serdes-a88c9aec01a6</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -9170,7 +9176,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>5.1.1-model-abi_in-8daf81be376d</t>
+          <t>5.1.1-model-abi_in-8462bca9d441</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -9239,7 +9245,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>5.2.6-model-abi_in-ffb26e2a6c06</t>
+          <t>5.2.6-model-abi_in-c0d5b5927261</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -9306,7 +9312,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>5.2.8-model-abi_in-5b18a46e1e28</t>
+          <t>5.2.8-model-abi_in-a5cd41b680d3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -9373,7 +9379,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>5.5.2-model-abi_in-c90c6b4a570b</t>
+          <t>5.5.2-model-abi_in-364e91a61d1b</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -9440,7 +9446,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>5.1.1-model-abi_out-a0b2eee78e2b</t>
+          <t>5.1.1-model-abi_out-d547c675a718</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -9509,7 +9515,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>5.2.6-model-abi_out-abe3dacb97d2</t>
+          <t>5.2.6-model-abi_out-9616478fba87</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9576,7 +9582,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>5.2.8-model-abi_out-bb5f806fc07b</t>
+          <t>5.2.8-model-abi_out-05564a97902a</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -9643,7 +9649,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>5.5.2-model-abi_out-121439f46ca3</t>
+          <t>5.5.2-model-abi_out-b4d2c741b2d2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -9711,7 +9717,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>5.1.1-model-refclk-3e0a1b16e22e</t>
+          <t>5.1.1-model-refclk-0acd87da3e4f</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9780,7 +9786,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>5.2.6-model-refclk-60f97d48d065</t>
+          <t>5.2.6-model-refclk-5e7292d2455e</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9847,7 +9853,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>5.2.8-model-refclk-b4e1f130aea0</t>
+          <t>5.2.8-model-refclk-e4e82d2ca84d</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -9914,7 +9920,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5.5.2-model-refclk-6086ef700a41</t>
+          <t>5.5.2-model-refclk-375978077e47</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9981,7 +9987,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5.1.2-model-abi_in-1b0f42a88c58</t>
+          <t>5.1.2-model-abi_in-9d5c4c99fd28</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -10048,7 +10054,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5.1.4-model-abi_in-04e8780cc1ea</t>
+          <t>5.1.4-model-abi_in-325704e4053d</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -10119,7 +10125,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5.3.6-model-abi_in-223e3fc544af</t>
+          <t>5.3.6-model-abi_in-4ae63af6ec4c</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -10186,7 +10192,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5.3.14-model-abi_in-bc009e4cbea5</t>
+          <t>5.3.14-model-abi_in-26ead24b2b6f</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -10253,7 +10259,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5.3.10-model-abi_in-dd40b7f19e81</t>
+          <t>5.3.10-model-abi_in-f65a468ac348</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -10320,7 +10326,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5.4.1-model-abi_in-886257d8e071</t>
+          <t>5.4.1-model-abi_in-29f8feda84cb</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -10387,7 +10393,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>5.4.2-model-abi_in-9412f9fb8a50</t>
+          <t>5.4.2-model-abi_in-c3dbf739ba6c</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -10454,7 +10460,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5.4.3-model-abi_in-b076a9650e86</t>
+          <t>5.4.3-model-abi_in-e0754c7fb43b</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -10521,7 +10527,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5.4.4-model-abi_in-6db97baec051</t>
+          <t>5.4.4-model-abi_in-70acd5ffa015</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -10588,7 +10594,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5.5.4-model-abi_in-154891a14567</t>
+          <t>5.5.4-model-abi_in-e0fc51f36f24</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -10655,7 +10661,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>5.6.2-model-abi_in-31ef5b9073c9</t>
+          <t>5.6.2-model-abi_in-a0f4fb0cccba</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -10722,7 +10728,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5.1.2-model-abi_out-c1641fff38b7</t>
+          <t>5.1.2-model-abi_out-a6cd2a20a114</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -10789,7 +10795,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5.1.4-model-abi_out-2799277fbe81</t>
+          <t>5.1.4-model-abi_out-de25ce796de4</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -10860,7 +10866,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>5.3.6-model-abi_out-0afe2e981ed4</t>
+          <t>5.3.6-model-abi_out-0312c5445aa8</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -10928,7 +10934,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>5.3.14-model-abi_out-c4637e606656</t>
+          <t>5.3.14-model-abi_out-845ca2889b33</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -10996,7 +11002,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5.3.10-model-abi_out-0c215bb8b564</t>
+          <t>5.3.10-model-abi_out-9271b77a393f</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -11063,7 +11069,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>5.4.1-model-abi_out-c5963c61a9e4</t>
+          <t>5.4.1-model-abi_out-49e68cecbdd0</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -11130,7 +11136,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>5.4.2-model-abi_out-b1a7443cb13d</t>
+          <t>5.4.2-model-abi_out-1adc8b663db2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -11197,7 +11203,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>5.4.3-model-abi_out-1a559536d201</t>
+          <t>5.4.3-model-abi_out-e3c2d6271733</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -11264,7 +11270,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>5.4.4-model-abi_out-7fbdcfbed324</t>
+          <t>5.4.4-model-abi_out-86d3ef4f058b</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -11331,7 +11337,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>5.5.4-model-abi_out-3103f02a8e44</t>
+          <t>5.5.4-model-abi_out-cf68cd0c8623</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -11398,7 +11404,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>5.6.2-model-abi_out-49dea042c996</t>
+          <t>5.6.2-model-abi_out-6ffdf871b1d1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -11465,7 +11471,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>5.1.2-model-refclk-331b017357e7</t>
+          <t>5.1.2-model-refclk-880011bb732d</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -11532,7 +11538,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>5.1.4-model-refclk-608360373a99</t>
+          <t>5.1.4-model-refclk-765445eea6f6</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -11603,7 +11609,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>5.3.6-model-refclk-f066bf7331f7</t>
+          <t>5.3.6-model-refclk-184019c27308</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -11670,7 +11676,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>5.3.14-model-refclk-a2fe2435361a</t>
+          <t>5.3.14-model-refclk-60889f484433</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -11737,7 +11743,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>5.3.10-model-refclk-15f56f936e4c</t>
+          <t>5.3.10-model-refclk-b34e4466fec9</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -11805,7 +11811,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>5.4.1-model-refclk-726a3e764243</t>
+          <t>5.4.1-model-refclk-b773e9e4fb34</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -11872,7 +11878,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>5.4.2-model-refclk-9bbc61c1ac58</t>
+          <t>5.4.2-model-refclk-3c4b9bc639a2</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -11939,7 +11945,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>5.4.3-model-refclk-9017c9b44d8e</t>
+          <t>5.4.3-model-refclk-241f6ca99193</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -12006,7 +12012,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>5.4.4-model-refclk-c2c6595d0387</t>
+          <t>5.4.4-model-refclk-4e0b2be9f45d</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -12073,7 +12079,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>5.5.4-model-refclk-2187eec3eda4</t>
+          <t>5.5.4-model-refclk-8ef78f283450</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -12140,7 +12146,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>5.6.2-model-refclk-51690742dcd6</t>
+          <t>5.6.2-model-refclk-0135fff3c7b9</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -12207,7 +12213,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>5.3.1-model-abi_in-742f786d8e5b</t>
+          <t>5.3.1-model-abi_in-e501a9f076ae</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -12274,7 +12280,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>5.3.2-model-abi_in-c112a75a1c43</t>
+          <t>5.3.2-model-abi_in-984f0b7824ba</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -12341,7 +12347,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>5.3.3-model-abi_in-1e7db9bbcc51</t>
+          <t>5.3.3-model-abi_in-3e2086a79ee0</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -12408,7 +12414,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>5.3.5-model-abi_in-bc2e0ff6c951</t>
+          <t>5.3.5-model-abi_in-fdef3bff78ce</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -12475,7 +12481,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>5.3.7-model-abi_in-69407e454ffa</t>
+          <t>5.3.7-model-abi_in-d771eaa4ee01</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -12542,7 +12548,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>5.3.8-model-abi_in-96bedb816555</t>
+          <t>5.3.8-model-abi_in-2278f8f6aca4</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -12609,7 +12615,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>5.3.9-model-abi_in-b90b0c4abf01</t>
+          <t>5.3.9-model-abi_in-16ed0211d5a5</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -12676,7 +12682,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>5.3.1-model-abi_out-c203504a7324</t>
+          <t>5.3.1-model-abi_out-48865479bd60</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -12743,7 +12749,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>5.3.1-model-abi_out-4ef437cf41b5</t>
+          <t>5.3.1-model-abi_out-48865479bd60-2</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -12810,7 +12816,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>5.3.2-model-abi_out-9db2c6bbf2c9</t>
+          <t>5.3.2-model-abi_out-e86abd88a25a</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -12877,7 +12883,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>5.3.3-model-abi_out-3599495e1f36</t>
+          <t>5.3.3-model-abi_out-932d1c3bd197</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -12944,7 +12950,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>5.3.7-model-abi_out-c9b4be37a73f</t>
+          <t>5.3.7-model-abi_out-8eeeddf99614</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -13011,7 +13017,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>5.3.7-model-abi_out-a1cda94dad4a</t>
+          <t>5.3.7-model-abi_out-8eeeddf99614-2</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -13078,7 +13084,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>5.3.8-model-abi_out-b98ea9dd8c8b</t>
+          <t>5.3.8-model-abi_out-c7faf5af1743</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -13145,7 +13151,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>5.3.9-model-abi_out-0a82d52d1945</t>
+          <t>5.3.9-model-abi_out-c8415a71fb80</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -13212,7 +13218,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>5.3.1-model-refclk-ec1b088b97ac</t>
+          <t>5.3.1-model-refclk-fc676a9a0070</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -13279,7 +13285,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>5.3.1-model-refclk-ea8125fa8cf9</t>
+          <t>5.3.1-model-refclk-fc676a9a0070-2</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -13346,7 +13352,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>5.3.2-model-refclk-238bff1b96a3</t>
+          <t>5.3.2-model-refclk-2fff1f6f19f8</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -13413,7 +13419,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>5.3.3-model-refclk-3dcd9f40ad9b</t>
+          <t>5.3.3-model-refclk-1ffd548c76f7</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -13480,7 +13486,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>5.3.4-model-refclk-d9d5c57de3c7</t>
+          <t>5.3.4-model-refclk-6a67590ca5b8</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -13547,7 +13553,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>5.3.5-model-refclk-7f25a270b5c0</t>
+          <t>5.3.5-model-refclk-9e67566e4de0</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -13614,7 +13620,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>5.3.7-model-refclk-39d382ab9f31</t>
+          <t>5.3.7-model-refclk-e279f6b70816</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -13681,7 +13687,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>5.3.7-model-refclk-eff48e020ec0</t>
+          <t>5.3.7-model-refclk-e279f6b70816-2</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -13748,7 +13754,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>5.3.8-model-refclk-a03f964429bf</t>
+          <t>5.3.8-model-refclk-221bbf6ccada</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -13815,7 +13821,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>5.3.9-model-refclk-3f97b9d8d956</t>
+          <t>5.3.9-model-refclk-215ae32ac881</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -13882,7 +13888,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>5.5.1-model-abi_out-34f5c53ce320</t>
+          <t>5.5.1-model-abi_out-03f0b1beea0e</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -13949,7 +13955,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>5.5.3-model-abi_out-a15d762f2ada</t>
+          <t>5.5.3-model-abi_out-2b81d06be3bd</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -14024,6 +14030,207 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>5.9.1-model-abi_in-daa3aef6cbae</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>5.9.1</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>LEVEL 2</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr" s="7">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr" s="7">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>abi_in</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Model_type=Input has no Pullup/Pulldown — Zout NA</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>5.9.1-model-abi_out-fab9cfcc7ab2</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>5.9.1</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>LEVEL 2</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr" s="4">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr" s="4">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>abi_out</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Zout worst-case 57.5Ω within 100Ω threshold</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>5.9.1-model-refclk-e609345acb2a</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>5.9.1</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>LEVEL 2</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr" s="7">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr" s="7">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>refclk</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Model_type=Input has no Pullup/Pulldown — Zout NA</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>